<commit_message>
feat: update REQ-07 and TC-07 to include harmful gas detection and environment monitoring
</commit_message>
<xml_diff>
--- a/Phytium_PPE_System_SourceCode/功能测试表.xlsx
+++ b/Phytium_PPE_System_SourceCode/功能测试表.xlsx
@@ -1626,7 +1626,7 @@
       </c>
       <c r="F12" s="36" t="n"/>
     </row>
-    <row r="13" ht="46" customFormat="1" customHeight="1" s="2">
+    <row r="13" ht="63" customFormat="1" customHeight="1" s="2">
       <c r="A13" s="34" t="inlineStr">
         <is>
           <t>TC-07</t>
@@ -1634,43 +1634,43 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>软硬联动模块</t>
+          <t>软硬联动与环境检测</t>
         </is>
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
           <t>1. OpenAMP 底层通信链路已就绪。
-2. 主核处于 AI 推理满载状态。</t>
+2. 从核已接入火焰、有害气体及温湿度传感器并满载运行。</t>
         </is>
       </c>
       <c r="D13" s="35" t="inlineStr">
         <is>
-          <t>1. 物理触发火焰传感器，向从核注入低电平硬件中断。</t>
+          <t>1. 物理触发火焰与有害气体传感器，向从核注入硬件中断与 ADC 模拟数据。</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>1. rx_task 极速捕获中断并完成 UI 渲染，端到端延迟 &lt; 20ms。</t>
+          <t>1. rx_task 极速捕获中断并渲染 UI，报警端到端延迟 &lt; 20ms，有害气体 ADC 采样值精准。</t>
         </is>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
-          <t>Pass。火焰传感器硬中断抢占机制测试通过。在 50ms 模拟抖动下未触发误报，Qt 界面火警弹窗显示稳定。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="29" customFormat="1" customHeight="1" s="2">
+          <t>Pass。火焰与有害气体硬中断抢占机制测试通过。在 50ms 模拟抖动下无闪烁；温湿度环境数据大屏实时刷新无误。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customFormat="1" customHeight="1" s="2">
       <c r="A14" s="36" t="n"/>
       <c r="B14" s="36" t="n"/>
       <c r="C14" s="36" t="n"/>
       <c r="D14" s="35" t="inlineStr">
         <is>
-          <t>2. 模拟 50ms 内的临界电平抖动，观察界面稳定性。</t>
+          <t>2. 模拟 50ms 内的临界电平抖动，并读取 AHT20 温湿度传感器数据，观察界面显示。</t>
         </is>
       </c>
       <c r="E14" s="35" t="inlineStr">
         <is>
-          <t>2. 排除抖动干扰，UI 报警状态锁定 500ms 后重置，无闪烁。</t>
+          <t>2. 排除抖动干扰，报警状态锁定 500ms 后重置，温湿度环境数据大屏每 2s 稳定刷新，无闪烁现象。</t>
         </is>
       </c>
       <c r="F14" s="36" t="n"/>
@@ -1877,7 +1877,7 @@
       <c r="E21" s="35" t="inlineStr">
         <is>
           <t>1. 心跳中断 2s 后从核接管并拉高 GPIO 驱动蜂鸣器长鸣报警，同时停止向 WDT 喂狗。
-2. 停止喂狗 10s 后 WDT 超时溢出，硬件强制复位芯片 cold reset 冷重启系统。</t>
+2. 停止喂狗 10s 后 WDT 超时溢出，硬件强制复位芯片冷重启系统。</t>
         </is>
       </c>
       <c r="F21" s="34" t="inlineStr">

</xml_diff>